<commit_message>
fix CI compiler job: resolve artifact subdirectory layout and default wrap imports
</commit_message>
<xml_diff>
--- a/dist-test/appium-android-report.xlsx
+++ b/dist-test/appium-android-report.xlsx
@@ -410,7 +410,7 @@
         <v>Generated on:</v>
       </c>
       <c r="B2" t="str">
-        <v>22/6/2026, 2:17:48 pm</v>
+        <v>22/6/2026, 2:30:09 pm</v>
       </c>
     </row>
     <row r="4">
@@ -559,7 +559,7 @@
         <v>PASS</v>
       </c>
       <c r="H2">
-        <v>62</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -585,7 +585,7 @@
         <v>PASS</v>
       </c>
       <c r="H3">
-        <v>35</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -611,7 +611,7 @@
         <v>PASS</v>
       </c>
       <c r="H4">
-        <v>23</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
@@ -637,7 +637,7 @@
         <v>PASS</v>
       </c>
       <c r="H5">
-        <v>84</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -663,7 +663,7 @@
         <v>PASS</v>
       </c>
       <c r="H6">
-        <v>101</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7">
@@ -689,7 +689,7 @@
         <v>PASS</v>
       </c>
       <c r="H7">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">
@@ -715,7 +715,7 @@
         <v>PASS</v>
       </c>
       <c r="H8">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9">
@@ -741,7 +741,7 @@
         <v>PASS</v>
       </c>
       <c r="H9">
-        <v>26</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10">
@@ -767,7 +767,7 @@
         <v>PASS</v>
       </c>
       <c r="H10">
-        <v>41</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
@@ -793,7 +793,7 @@
         <v>PASS</v>
       </c>
       <c r="H11">
-        <v>77</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
@@ -819,7 +819,7 @@
         <v>PASS</v>
       </c>
       <c r="H12">
-        <v>58</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13">
@@ -845,7 +845,7 @@
         <v>PASS</v>
       </c>
       <c r="H13">
-        <v>68</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -871,7 +871,7 @@
         <v>PASS</v>
       </c>
       <c r="H14">
-        <v>24</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15">
@@ -897,7 +897,7 @@
         <v>PASS</v>
       </c>
       <c r="H15">
-        <v>50</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16">
@@ -923,7 +923,7 @@
         <v>PASS</v>
       </c>
       <c r="H16">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17">
@@ -949,7 +949,7 @@
         <v>PASS</v>
       </c>
       <c r="H17">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
@@ -975,7 +975,7 @@
         <v>PASS</v>
       </c>
       <c r="H18">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
@@ -1001,7 +1001,7 @@
         <v>PASS</v>
       </c>
       <c r="H19">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -1027,7 +1027,7 @@
         <v>PASS</v>
       </c>
       <c r="H20">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -1053,7 +1053,7 @@
         <v>PASS</v>
       </c>
       <c r="H21">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -1079,7 +1079,7 @@
         <v>PASS</v>
       </c>
       <c r="H22">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -1105,7 +1105,7 @@
         <v>PASS</v>
       </c>
       <c r="H23">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -1209,7 +1209,7 @@
         <v>PASS</v>
       </c>
       <c r="H27">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
@@ -1235,7 +1235,7 @@
         <v>PASS</v>
       </c>
       <c r="H28">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29">
@@ -1261,7 +1261,7 @@
         <v>PASS</v>
       </c>
       <c r="H29">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -1287,7 +1287,7 @@
         <v>PASS</v>
       </c>
       <c r="H30">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31">
@@ -1339,7 +1339,7 @@
         <v>PASS</v>
       </c>
       <c r="H32">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -1365,7 +1365,7 @@
         <v>PASS</v>
       </c>
       <c r="H33">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -1417,7 +1417,7 @@
         <v>PASS</v>
       </c>
       <c r="H35">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36">
@@ -1443,7 +1443,7 @@
         <v>PASS</v>
       </c>
       <c r="H36">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
@@ -1495,7 +1495,7 @@
         <v>PASS</v>
       </c>
       <c r="H38">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39">
@@ -1521,7 +1521,7 @@
         <v>PASS</v>
       </c>
       <c r="H39">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40">
@@ -1573,7 +1573,7 @@
         <v>PASS</v>
       </c>
       <c r="H41">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="42">
@@ -1599,7 +1599,7 @@
         <v>PASS</v>
       </c>
       <c r="H42">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
@@ -1625,7 +1625,7 @@
         <v>PASS</v>
       </c>
       <c r="H43">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="44">
@@ -1651,7 +1651,7 @@
         <v>PASS</v>
       </c>
       <c r="H44">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45">
@@ -1677,7 +1677,7 @@
         <v>PASS</v>
       </c>
       <c r="H45">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
@@ -1729,7 +1729,7 @@
         <v>PASS</v>
       </c>
       <c r="H47">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="48">
@@ -1755,7 +1755,7 @@
         <v>PASS</v>
       </c>
       <c r="H48">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="49">
@@ -1781,7 +1781,7 @@
         <v>PASS</v>
       </c>
       <c r="H49">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50">
@@ -1807,7 +1807,7 @@
         <v>PASS</v>
       </c>
       <c r="H50">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51">
@@ -1833,7 +1833,7 @@
         <v>PASS</v>
       </c>
       <c r="H51">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52">
@@ -1859,7 +1859,7 @@
         <v>PASS</v>
       </c>
       <c r="H52">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53">
@@ -1885,7 +1885,7 @@
         <v>PASS</v>
       </c>
       <c r="H53">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="54">
@@ -1911,7 +1911,7 @@
         <v>PASS</v>
       </c>
       <c r="H54">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55">
@@ -1937,7 +1937,7 @@
         <v>PASS</v>
       </c>
       <c r="H55">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="56">
@@ -1963,7 +1963,7 @@
         <v>PASS</v>
       </c>
       <c r="H56">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="57">
@@ -1989,7 +1989,7 @@
         <v>PASS</v>
       </c>
       <c r="H57">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="58">
@@ -2015,7 +2015,7 @@
         <v>PASS</v>
       </c>
       <c r="H58">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59">
@@ -2041,7 +2041,7 @@
         <v>PASS</v>
       </c>
       <c r="H59">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="60">
@@ -2067,7 +2067,7 @@
         <v>PASS</v>
       </c>
       <c r="H60">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="61">
@@ -2093,7 +2093,7 @@
         <v>PASS</v>
       </c>
       <c r="H61">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="62">
@@ -2119,7 +2119,7 @@
         <v>PASS</v>
       </c>
       <c r="H62">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63">
@@ -2145,7 +2145,7 @@
         <v>PASS</v>
       </c>
       <c r="H63">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="64">
@@ -2171,7 +2171,7 @@
         <v>PASS</v>
       </c>
       <c r="H64">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="65">
@@ -2197,7 +2197,7 @@
         <v>PASS</v>
       </c>
       <c r="H65">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="66">
@@ -2223,7 +2223,7 @@
         <v>PASS</v>
       </c>
       <c r="H66">
-        <v>9</v>
+        <v>23</v>
       </c>
     </row>
     <row r="67">
@@ -2249,7 +2249,7 @@
         <v>PASS</v>
       </c>
       <c r="H67">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="68">
@@ -2275,7 +2275,7 @@
         <v>PASS</v>
       </c>
       <c r="H68">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69">
@@ -2301,7 +2301,7 @@
         <v>PASS</v>
       </c>
       <c r="H69">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70">
@@ -2327,7 +2327,7 @@
         <v>PASS</v>
       </c>
       <c r="H70">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="71">
@@ -2379,7 +2379,7 @@
         <v>PASS</v>
       </c>
       <c r="H72">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="73">
@@ -2405,7 +2405,7 @@
         <v>PASS</v>
       </c>
       <c r="H73">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="74">
@@ -2431,7 +2431,7 @@
         <v>PASS</v>
       </c>
       <c r="H74">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="75">
@@ -2457,7 +2457,7 @@
         <v>PASS</v>
       </c>
       <c r="H75">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="76">
@@ -2483,7 +2483,7 @@
         <v>PASS</v>
       </c>
       <c r="H76">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77">
@@ -2509,7 +2509,7 @@
         <v>PASS</v>
       </c>
       <c r="H77">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78">
@@ -2535,7 +2535,7 @@
         <v>PASS</v>
       </c>
       <c r="H78">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79">
@@ -2561,7 +2561,7 @@
         <v>PASS</v>
       </c>
       <c r="H79">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="80">
@@ -2587,7 +2587,7 @@
         <v>PASS</v>
       </c>
       <c r="H80">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="81">
@@ -2613,7 +2613,7 @@
         <v>PASS</v>
       </c>
       <c r="H81">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="82">
@@ -2639,7 +2639,7 @@
         <v>PASS</v>
       </c>
       <c r="H82">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="83">
@@ -2665,7 +2665,7 @@
         <v>PASS</v>
       </c>
       <c r="H83">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="84">
@@ -2717,7 +2717,7 @@
         <v>PASS</v>
       </c>
       <c r="H85">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
     <row r="86">
@@ -2743,7 +2743,7 @@
         <v>PASS</v>
       </c>
       <c r="H86">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="87">
@@ -2769,7 +2769,7 @@
         <v>PASS</v>
       </c>
       <c r="H87">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88">
@@ -2795,7 +2795,7 @@
         <v>PASS</v>
       </c>
       <c r="H88">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="89">
@@ -2821,7 +2821,7 @@
         <v>PASS</v>
       </c>
       <c r="H89">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90">
@@ -2847,7 +2847,7 @@
         <v>PASS</v>
       </c>
       <c r="H90">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="91">
@@ -2873,7 +2873,7 @@
         <v>PASS</v>
       </c>
       <c r="H91">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="92">
@@ -2899,7 +2899,7 @@
         <v>PASS</v>
       </c>
       <c r="H92">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="93">
@@ -2925,7 +2925,7 @@
         <v>PASS</v>
       </c>
       <c r="H93">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="94">
@@ -2951,7 +2951,7 @@
         <v>PASS</v>
       </c>
       <c r="H94">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="95">
@@ -2977,7 +2977,7 @@
         <v>PASS</v>
       </c>
       <c r="H95">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="96">
@@ -3003,7 +3003,7 @@
         <v>PASS</v>
       </c>
       <c r="H96">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="97">
@@ -3029,7 +3029,7 @@
         <v>PASS</v>
       </c>
       <c r="H97">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="98">
@@ -3055,7 +3055,7 @@
         <v>PASS</v>
       </c>
       <c r="H98">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="99">
@@ -3081,7 +3081,7 @@
         <v>PASS</v>
       </c>
       <c r="H99">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="100">
@@ -3107,7 +3107,7 @@
         <v>PASS</v>
       </c>
       <c r="H100">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="101">
@@ -3133,7 +3133,7 @@
         <v>PASS</v>
       </c>
       <c r="H101">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="102">
@@ -3159,7 +3159,7 @@
         <v>PASS</v>
       </c>
       <c r="H102">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="103">
@@ -3185,7 +3185,7 @@
         <v>PASS</v>
       </c>
       <c r="H103">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="104">
@@ -3211,7 +3211,7 @@
         <v>PASS</v>
       </c>
       <c r="H104">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="105">
@@ -3237,7 +3237,7 @@
         <v>PASS</v>
       </c>
       <c r="H105">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="106">
@@ -3263,7 +3263,7 @@
         <v>PASS</v>
       </c>
       <c r="H106">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="107">
@@ -3289,7 +3289,7 @@
         <v>PASS</v>
       </c>
       <c r="H107">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="108">
@@ -3315,7 +3315,7 @@
         <v>PASS</v>
       </c>
       <c r="H108">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="109">
@@ -3341,7 +3341,7 @@
         <v>PASS</v>
       </c>
       <c r="H109">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="110">
@@ -3367,7 +3367,7 @@
         <v>PASS</v>
       </c>
       <c r="H110">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111">
@@ -3393,7 +3393,7 @@
         <v>PASS</v>
       </c>
       <c r="H111">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="112">
@@ -3419,7 +3419,7 @@
         <v>PASS</v>
       </c>
       <c r="H112">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="113">
@@ -3445,7 +3445,7 @@
         <v>PASS</v>
       </c>
       <c r="H113">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="114">
@@ -3471,7 +3471,7 @@
         <v>PASS</v>
       </c>
       <c r="H114">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="115">
@@ -3497,7 +3497,7 @@
         <v>PASS</v>
       </c>
       <c r="H115">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="116">
@@ -3523,7 +3523,7 @@
         <v>PASS</v>
       </c>
       <c r="H116">
-        <v>14</v>
+        <v>32</v>
       </c>
     </row>
     <row r="117">
@@ -3549,7 +3549,7 @@
         <v>PASS</v>
       </c>
       <c r="H117">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="118">
@@ -3575,7 +3575,7 @@
         <v>PASS</v>
       </c>
       <c r="H118">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="119">
@@ -3601,7 +3601,7 @@
         <v>PASS</v>
       </c>
       <c r="H119">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="120">
@@ -3627,7 +3627,7 @@
         <v>PASS</v>
       </c>
       <c r="H120">
-        <v>31</v>
+        <v>9</v>
       </c>
     </row>
     <row r="121">
@@ -3653,7 +3653,7 @@
         <v>PASS</v>
       </c>
       <c r="H121">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="122">
@@ -3679,7 +3679,7 @@
         <v>PASS</v>
       </c>
       <c r="H122">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="123">
@@ -3705,7 +3705,7 @@
         <v>PASS</v>
       </c>
       <c r="H123">
-        <v>29</v>
+        <v>9</v>
       </c>
     </row>
     <row r="124">
@@ -3731,7 +3731,7 @@
         <v>PASS</v>
       </c>
       <c r="H124">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="125">
@@ -3757,7 +3757,7 @@
         <v>PASS</v>
       </c>
       <c r="H125">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="126">
@@ -3783,7 +3783,7 @@
         <v>PASS</v>
       </c>
       <c r="H126">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="127">
@@ -3809,7 +3809,7 @@
         <v>PASS</v>
       </c>
       <c r="H127">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="128">
@@ -3835,7 +3835,7 @@
         <v>PASS</v>
       </c>
       <c r="H128">
-        <v>14</v>
+        <v>29</v>
       </c>
     </row>
     <row r="129">
@@ -3861,7 +3861,7 @@
         <v>PASS</v>
       </c>
       <c r="H129">
-        <v>16</v>
+        <v>31</v>
       </c>
     </row>
     <row r="130">
@@ -3887,7 +3887,7 @@
         <v>PASS</v>
       </c>
       <c r="H130">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="131">
@@ -3913,7 +3913,7 @@
         <v>PASS</v>
       </c>
       <c r="H131">
-        <v>31</v>
+        <v>8</v>
       </c>
     </row>
     <row r="132">
@@ -3939,7 +3939,7 @@
         <v>PASS</v>
       </c>
       <c r="H132">
-        <v>32</v>
+        <v>9</v>
       </c>
     </row>
     <row r="133">
@@ -3965,7 +3965,7 @@
         <v>PASS</v>
       </c>
       <c r="H133">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="134">
@@ -3991,7 +3991,7 @@
         <v>PASS</v>
       </c>
       <c r="H134">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="135">
@@ -4017,7 +4017,7 @@
         <v>PASS</v>
       </c>
       <c r="H135">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="136">
@@ -4043,7 +4043,7 @@
         <v>PASS</v>
       </c>
       <c r="H136">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="137">
@@ -4069,7 +4069,7 @@
         <v>PASS</v>
       </c>
       <c r="H137">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="138">
@@ -4095,7 +4095,7 @@
         <v>PASS</v>
       </c>
       <c r="H138">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="139">
@@ -4121,7 +4121,7 @@
         <v>PASS</v>
       </c>
       <c r="H139">
-        <v>9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="140">
@@ -4147,7 +4147,7 @@
         <v>PASS</v>
       </c>
       <c r="H140">
-        <v>27</v>
+        <v>13</v>
       </c>
     </row>
     <row r="141">
@@ -4173,7 +4173,7 @@
         <v>PASS</v>
       </c>
       <c r="H141">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="142">
@@ -4199,7 +4199,7 @@
         <v>PASS</v>
       </c>
       <c r="H142">
-        <v>29</v>
+        <v>8</v>
       </c>
     </row>
     <row r="143">
@@ -4225,7 +4225,7 @@
         <v>PASS</v>
       </c>
       <c r="H143">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="144">
@@ -4251,7 +4251,7 @@
         <v>PASS</v>
       </c>
       <c r="H144">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="145">
@@ -4277,7 +4277,7 @@
         <v>PASS</v>
       </c>
       <c r="H145">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="146">
@@ -4303,7 +4303,7 @@
         <v>PASS</v>
       </c>
       <c r="H146">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="147">
@@ -4329,7 +4329,7 @@
         <v>PASS</v>
       </c>
       <c r="H147">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="148">
@@ -4355,7 +4355,7 @@
         <v>PASS</v>
       </c>
       <c r="H148">
-        <v>17</v>
+        <v>26</v>
       </c>
     </row>
     <row r="149">
@@ -4381,7 +4381,7 @@
         <v>PASS</v>
       </c>
       <c r="H149">
-        <v>10</v>
+        <v>31</v>
       </c>
     </row>
     <row r="150">
@@ -4407,7 +4407,7 @@
         <v>PASS</v>
       </c>
       <c r="H150">
-        <v>26</v>
+        <v>11</v>
       </c>
     </row>
     <row r="151">
@@ -4433,7 +4433,7 @@
         <v>PASS</v>
       </c>
       <c r="H151">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="152">
@@ -4459,7 +4459,7 @@
         <v>PASS</v>
       </c>
       <c r="H152">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="153">
@@ -4485,7 +4485,7 @@
         <v>PASS</v>
       </c>
       <c r="H153">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="154">
@@ -4511,7 +4511,7 @@
         <v>PASS</v>
       </c>
       <c r="H154">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="155">
@@ -4537,7 +4537,7 @@
         <v>PASS</v>
       </c>
       <c r="H155">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="156">
@@ -4563,7 +4563,7 @@
         <v>PASS</v>
       </c>
       <c r="H156">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="157">
@@ -4589,7 +4589,7 @@
         <v>PASS</v>
       </c>
       <c r="H157">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="158">
@@ -4615,7 +4615,7 @@
         <v>PASS</v>
       </c>
       <c r="H158">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="159">
@@ -4641,7 +4641,7 @@
         <v>PASS</v>
       </c>
       <c r="H159">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="160">
@@ -4667,7 +4667,7 @@
         <v>PASS</v>
       </c>
       <c r="H160">
-        <v>14</v>
+        <v>25</v>
       </c>
     </row>
     <row r="161">
@@ -4693,7 +4693,7 @@
         <v>PASS</v>
       </c>
       <c r="H161">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="162">
@@ -4719,7 +4719,7 @@
         <v>PASS</v>
       </c>
       <c r="H162">
-        <v>31</v>
+        <v>12</v>
       </c>
     </row>
     <row r="163">
@@ -4745,7 +4745,7 @@
         <v>PASS</v>
       </c>
       <c r="H163">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="164">
@@ -4771,7 +4771,7 @@
         <v>PASS</v>
       </c>
       <c r="H164">
-        <v>11</v>
+        <v>28</v>
       </c>
     </row>
     <row r="165">
@@ -4797,7 +4797,7 @@
         <v>PASS</v>
       </c>
       <c r="H165">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="166">
@@ -4823,7 +4823,7 @@
         <v>PASS</v>
       </c>
       <c r="H166">
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
     <row r="167">
@@ -4849,7 +4849,7 @@
         <v>PASS</v>
       </c>
       <c r="H167">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="168">
@@ -4875,7 +4875,7 @@
         <v>PASS</v>
       </c>
       <c r="H168">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="169">
@@ -4901,7 +4901,7 @@
         <v>PASS</v>
       </c>
       <c r="H169">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="170">
@@ -4927,7 +4927,7 @@
         <v>PASS</v>
       </c>
       <c r="H170">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="171">
@@ -4953,7 +4953,7 @@
         <v>PASS</v>
       </c>
       <c r="H171">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="172">
@@ -4979,7 +4979,7 @@
         <v>PASS</v>
       </c>
       <c r="H172">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="173">
@@ -5005,7 +5005,7 @@
         <v>PASS</v>
       </c>
       <c r="H173">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="174">
@@ -5031,7 +5031,7 @@
         <v>PASS</v>
       </c>
       <c r="H174">
-        <v>26</v>
+        <v>9</v>
       </c>
     </row>
     <row r="175">
@@ -5057,7 +5057,7 @@
         <v>PASS</v>
       </c>
       <c r="H175">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="176">
@@ -5083,7 +5083,7 @@
         <v>PASS</v>
       </c>
       <c r="H176">
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="177">
@@ -5109,7 +5109,7 @@
         <v>PASS</v>
       </c>
       <c r="H177">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="178">
@@ -5135,7 +5135,7 @@
         <v>PASS</v>
       </c>
       <c r="H178">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="179">
@@ -5161,7 +5161,7 @@
         <v>PASS</v>
       </c>
       <c r="H179">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="180">
@@ -5187,7 +5187,7 @@
         <v>PASS</v>
       </c>
       <c r="H180">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="181">
@@ -5213,7 +5213,7 @@
         <v>PASS</v>
       </c>
       <c r="H181">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="182">
@@ -5239,7 +5239,7 @@
         <v>PASS</v>
       </c>
       <c r="H182">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="183">
@@ -5265,7 +5265,7 @@
         <v>PASS</v>
       </c>
       <c r="H183">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="184">
@@ -5291,7 +5291,7 @@
         <v>PASS</v>
       </c>
       <c r="H184">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="185">
@@ -5317,7 +5317,7 @@
         <v>PASS</v>
       </c>
       <c r="H185">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="186">
@@ -5343,7 +5343,7 @@
         <v>PASS</v>
       </c>
       <c r="H186">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="187">
@@ -5369,7 +5369,7 @@
         <v>PASS</v>
       </c>
       <c r="H187">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="188">
@@ -5395,7 +5395,7 @@
         <v>PASS</v>
       </c>
       <c r="H188">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="189">
@@ -5421,7 +5421,7 @@
         <v>PASS</v>
       </c>
       <c r="H189">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="190">
@@ -5447,7 +5447,7 @@
         <v>PASS</v>
       </c>
       <c r="H190">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="191">
@@ -5473,7 +5473,7 @@
         <v>PASS</v>
       </c>
       <c r="H191">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="192">
@@ -5499,7 +5499,7 @@
         <v>PASS</v>
       </c>
       <c r="H192">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="193">
@@ -5525,7 +5525,7 @@
         <v>PASS</v>
       </c>
       <c r="H193">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="194">
@@ -5551,7 +5551,7 @@
         <v>PASS</v>
       </c>
       <c r="H194">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="195">
@@ -5577,7 +5577,7 @@
         <v>PASS</v>
       </c>
       <c r="H195">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="196">
@@ -5603,7 +5603,7 @@
         <v>PASS</v>
       </c>
       <c r="H196">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="197">
@@ -5629,7 +5629,7 @@
         <v>PASS</v>
       </c>
       <c r="H197">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="198">
@@ -5681,7 +5681,7 @@
         <v>PASS</v>
       </c>
       <c r="H199">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="200">
@@ -5707,7 +5707,7 @@
         <v>PASS</v>
       </c>
       <c r="H200">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="201">
@@ -5733,7 +5733,7 @@
         <v>PASS</v>
       </c>
       <c r="H201">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="202">
@@ -5759,7 +5759,7 @@
         <v>PASS</v>
       </c>
       <c r="H202">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="203">
@@ -5785,7 +5785,7 @@
         <v>PASS</v>
       </c>
       <c r="H203">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="204">
@@ -5811,7 +5811,7 @@
         <v>PASS</v>
       </c>
       <c r="H204">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="205">
@@ -5837,7 +5837,7 @@
         <v>PASS</v>
       </c>
       <c r="H205">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="206">
@@ -5863,7 +5863,7 @@
         <v>PASS</v>
       </c>
       <c r="H206">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="207">
@@ -5889,7 +5889,7 @@
         <v>PASS</v>
       </c>
       <c r="H207">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="208">
@@ -5915,7 +5915,7 @@
         <v>PASS</v>
       </c>
       <c r="H208">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="209">
@@ -5941,7 +5941,7 @@
         <v>PASS</v>
       </c>
       <c r="H209">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="210">
@@ -5993,7 +5993,7 @@
         <v>PASS</v>
       </c>
       <c r="H211">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="212">
@@ -6019,7 +6019,7 @@
         <v>PASS</v>
       </c>
       <c r="H212">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="213">
@@ -6097,7 +6097,7 @@
         <v>PASS</v>
       </c>
       <c r="H215">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="216">
@@ -6123,7 +6123,7 @@
         <v>PASS</v>
       </c>
       <c r="H216">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="217">
@@ -6149,7 +6149,7 @@
         <v>PASS</v>
       </c>
       <c r="H217">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="218">
@@ -6175,7 +6175,7 @@
         <v>PASS</v>
       </c>
       <c r="H218">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="219">
@@ -6201,7 +6201,7 @@
         <v>PASS</v>
       </c>
       <c r="H219">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="220">
@@ -6227,7 +6227,7 @@
         <v>PASS</v>
       </c>
       <c r="H220">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="221">
@@ -6253,7 +6253,7 @@
         <v>PASS</v>
       </c>
       <c r="H221">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="222">
@@ -6279,7 +6279,7 @@
         <v>PASS</v>
       </c>
       <c r="H222">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="223">
@@ -6305,7 +6305,7 @@
         <v>PASS</v>
       </c>
       <c r="H223">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="224">
@@ -6331,7 +6331,7 @@
         <v>PASS</v>
       </c>
       <c r="H224">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="225">
@@ -6357,7 +6357,7 @@
         <v>PASS</v>
       </c>
       <c r="H225">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="226">
@@ -6383,7 +6383,7 @@
         <v>PASS</v>
       </c>
       <c r="H226">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="227">
@@ -6409,7 +6409,7 @@
         <v>PASS</v>
       </c>
       <c r="H227">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="228">
@@ -6435,7 +6435,7 @@
         <v>PASS</v>
       </c>
       <c r="H228">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="229">
@@ -6487,7 +6487,7 @@
         <v>PASS</v>
       </c>
       <c r="H230">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="231">
@@ -6513,7 +6513,7 @@
         <v>PASS</v>
       </c>
       <c r="H231">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="232">
@@ -6539,7 +6539,7 @@
         <v>PASS</v>
       </c>
       <c r="H232">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="233">
@@ -6565,7 +6565,7 @@
         <v>PASS</v>
       </c>
       <c r="H233">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="234">
@@ -6591,7 +6591,7 @@
         <v>PASS</v>
       </c>
       <c r="H234">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="235">
@@ -6617,7 +6617,7 @@
         <v>PASS</v>
       </c>
       <c r="H235">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="236">
@@ -6643,7 +6643,7 @@
         <v>PASS</v>
       </c>
       <c r="H236">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="237">
@@ -6669,7 +6669,7 @@
         <v>PASS</v>
       </c>
       <c r="H237">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="238">
@@ -6695,7 +6695,7 @@
         <v>PASS</v>
       </c>
       <c r="H238">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="239">
@@ -6721,7 +6721,7 @@
         <v>PASS</v>
       </c>
       <c r="H239">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="240">
@@ -6747,7 +6747,7 @@
         <v>PASS</v>
       </c>
       <c r="H240">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="241">
@@ -6773,7 +6773,7 @@
         <v>PASS</v>
       </c>
       <c r="H241">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="242">
@@ -6799,7 +6799,7 @@
         <v>PASS</v>
       </c>
       <c r="H242">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="243">
@@ -6825,7 +6825,7 @@
         <v>PASS</v>
       </c>
       <c r="H243">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="244">
@@ -6851,7 +6851,7 @@
         <v>PASS</v>
       </c>
       <c r="H244">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="245">
@@ -6877,7 +6877,7 @@
         <v>PASS</v>
       </c>
       <c r="H245">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="246">
@@ -6903,7 +6903,7 @@
         <v>PASS</v>
       </c>
       <c r="H246">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="247">
@@ -6929,7 +6929,7 @@
         <v>PASS</v>
       </c>
       <c r="H247">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="248">
@@ -6955,7 +6955,7 @@
         <v>PASS</v>
       </c>
       <c r="H248">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="249">
@@ -6981,7 +6981,7 @@
         <v>PASS</v>
       </c>
       <c r="H249">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="250">
@@ -7033,7 +7033,7 @@
         <v>PASS</v>
       </c>
       <c r="H251">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="252">
@@ -7059,7 +7059,7 @@
         <v>PASS</v>
       </c>
       <c r="H252">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="253">
@@ -7085,7 +7085,7 @@
         <v>PASS</v>
       </c>
       <c r="H253">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="254">
@@ -7137,7 +7137,7 @@
         <v>PASS</v>
       </c>
       <c r="H255">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="256">
@@ -7163,7 +7163,7 @@
         <v>PASS</v>
       </c>
       <c r="H256">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="257">
@@ -7189,7 +7189,7 @@
         <v>PASS</v>
       </c>
       <c r="H257">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="258">
@@ -7215,7 +7215,7 @@
         <v>PASS</v>
       </c>
       <c r="H258">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="259">
@@ -7241,7 +7241,7 @@
         <v>PASS</v>
       </c>
       <c r="H259">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="260">
@@ -7267,7 +7267,7 @@
         <v>PASS</v>
       </c>
       <c r="H260">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="261">
@@ -7293,7 +7293,7 @@
         <v>PASS</v>
       </c>
       <c r="H261">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="262">
@@ -7319,7 +7319,7 @@
         <v>PASS</v>
       </c>
       <c r="H262">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="263">
@@ -7371,7 +7371,7 @@
         <v>PASS</v>
       </c>
       <c r="H264">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="265">
@@ -7397,7 +7397,7 @@
         <v>PASS</v>
       </c>
       <c r="H265">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="266">
@@ -7423,7 +7423,7 @@
         <v>PASS</v>
       </c>
       <c r="H266">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="267">
@@ -7449,7 +7449,7 @@
         <v>PASS</v>
       </c>
       <c r="H267">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="268">
@@ -7475,7 +7475,7 @@
         <v>PASS</v>
       </c>
       <c r="H268">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="269">
@@ -7501,7 +7501,7 @@
         <v>PASS</v>
       </c>
       <c r="H269">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="270">
@@ -7527,7 +7527,7 @@
         <v>PASS</v>
       </c>
       <c r="H270">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="271">
@@ -7553,7 +7553,7 @@
         <v>PASS</v>
       </c>
       <c r="H271">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="272">
@@ -7605,7 +7605,7 @@
         <v>PASS</v>
       </c>
       <c r="H273">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="274">
@@ -7631,7 +7631,7 @@
         <v>PASS</v>
       </c>
       <c r="H274">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="275">
@@ -7657,7 +7657,7 @@
         <v>PASS</v>
       </c>
       <c r="H275">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="276">
@@ -7683,7 +7683,7 @@
         <v>PASS</v>
       </c>
       <c r="H276">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="277">
@@ -7709,7 +7709,7 @@
         <v>PASS</v>
       </c>
       <c r="H277">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="278">
@@ -7735,7 +7735,7 @@
         <v>PASS</v>
       </c>
       <c r="H278">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="279">
@@ -7761,7 +7761,7 @@
         <v>PASS</v>
       </c>
       <c r="H279">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="280">
@@ -7787,7 +7787,7 @@
         <v>PASS</v>
       </c>
       <c r="H280">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="281">
@@ -7813,7 +7813,7 @@
         <v>PASS</v>
       </c>
       <c r="H281">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="282">
@@ -7839,7 +7839,7 @@
         <v>PASS</v>
       </c>
       <c r="H282">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="283">
@@ -7865,7 +7865,7 @@
         <v>PASS</v>
       </c>
       <c r="H283">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="284">
@@ -7891,7 +7891,7 @@
         <v>PASS</v>
       </c>
       <c r="H284">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="285">
@@ -7917,7 +7917,7 @@
         <v>PASS</v>
       </c>
       <c r="H285">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="286">
@@ -7969,7 +7969,7 @@
         <v>PASS</v>
       </c>
       <c r="H287">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="288">
@@ -7995,7 +7995,7 @@
         <v>PASS</v>
       </c>
       <c r="H288">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="289">
@@ -8021,7 +8021,7 @@
         <v>PASS</v>
       </c>
       <c r="H289">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="290">
@@ -8047,7 +8047,7 @@
         <v>PASS</v>
       </c>
       <c r="H290">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="291">
@@ -8073,7 +8073,7 @@
         <v>PASS</v>
       </c>
       <c r="H291">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="292">
@@ -8099,7 +8099,7 @@
         <v>PASS</v>
       </c>
       <c r="H292">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="293">
@@ -8125,7 +8125,7 @@
         <v>PASS</v>
       </c>
       <c r="H293">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="294">
@@ -8151,7 +8151,7 @@
         <v>PASS</v>
       </c>
       <c r="H294">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="295">
@@ -8177,7 +8177,7 @@
         <v>PASS</v>
       </c>
       <c r="H295">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="296">
@@ -8203,7 +8203,7 @@
         <v>PASS</v>
       </c>
       <c r="H296">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="297">
@@ -8229,7 +8229,7 @@
         <v>PASS</v>
       </c>
       <c r="H297">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="298">
@@ -8255,7 +8255,7 @@
         <v>PASS</v>
       </c>
       <c r="H298">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="299">
@@ -8281,7 +8281,7 @@
         <v>PASS</v>
       </c>
       <c r="H299">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="300">
@@ -8307,7 +8307,7 @@
         <v>PASS</v>
       </c>
       <c r="H300">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="301">
@@ -8333,7 +8333,7 @@
         <v>PASS</v>
       </c>
       <c r="H301">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="302">
@@ -8385,7 +8385,7 @@
         <v>PASS</v>
       </c>
       <c r="H303">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="304">
@@ -8411,7 +8411,7 @@
         <v>PASS</v>
       </c>
       <c r="H304">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="305">
@@ -8437,7 +8437,7 @@
         <v>PASS</v>
       </c>
       <c r="H305">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="306">
@@ -8463,7 +8463,7 @@
         <v>PASS</v>
       </c>
       <c r="H306">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="307">
@@ -8489,7 +8489,7 @@
         <v>PASS</v>
       </c>
       <c r="H307">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="308">
@@ -8567,7 +8567,7 @@
         <v>PASS</v>
       </c>
       <c r="H310">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="311">
@@ -8593,7 +8593,7 @@
         <v>PASS</v>
       </c>
       <c r="H311">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="312">
@@ -8619,7 +8619,7 @@
         <v>PASS</v>
       </c>
       <c r="H312">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="313">
@@ -8645,7 +8645,7 @@
         <v>PASS</v>
       </c>
       <c r="H313">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="314">
@@ -8671,7 +8671,7 @@
         <v>PASS</v>
       </c>
       <c r="H314">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="315">
@@ -8697,7 +8697,7 @@
         <v>PASS</v>
       </c>
       <c r="H315">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="316">
@@ -8723,7 +8723,7 @@
         <v>PASS</v>
       </c>
       <c r="H316">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="317">
@@ -8775,7 +8775,7 @@
         <v>PASS</v>
       </c>
       <c r="H318">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="319">
@@ -8801,7 +8801,7 @@
         <v>PASS</v>
       </c>
       <c r="H319">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="320">
@@ -8827,7 +8827,7 @@
         <v>PASS</v>
       </c>
       <c r="H320">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="321">
@@ -8853,7 +8853,7 @@
         <v>PASS</v>
       </c>
       <c r="H321">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="322">
@@ -8879,7 +8879,7 @@
         <v>PASS</v>
       </c>
       <c r="H322">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="323">
@@ -8931,7 +8931,7 @@
         <v>PASS</v>
       </c>
       <c r="H324">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="325">
@@ -8957,7 +8957,7 @@
         <v>PASS</v>
       </c>
       <c r="H325">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="326">
@@ -8983,7 +8983,7 @@
         <v>PASS</v>
       </c>
       <c r="H326">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="327">
@@ -9009,7 +9009,7 @@
         <v>PASS</v>
       </c>
       <c r="H327">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="328">
@@ -9035,7 +9035,7 @@
         <v>PASS</v>
       </c>
       <c r="H328">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="329">
@@ -9087,7 +9087,7 @@
         <v>PASS</v>
       </c>
       <c r="H330">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="331">
@@ -9113,7 +9113,7 @@
         <v>PASS</v>
       </c>
       <c r="H331">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="332">
@@ -9139,7 +9139,7 @@
         <v>PASS</v>
       </c>
       <c r="H332">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="333">
@@ -9165,7 +9165,7 @@
         <v>PASS</v>
       </c>
       <c r="H333">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="334">
@@ -9191,7 +9191,7 @@
         <v>PASS</v>
       </c>
       <c r="H334">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="335">
@@ -9217,7 +9217,7 @@
         <v>PASS</v>
       </c>
       <c r="H335">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="336">
@@ -9243,7 +9243,7 @@
         <v>PASS</v>
       </c>
       <c r="H336">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="337">
@@ -9269,7 +9269,7 @@
         <v>PASS</v>
       </c>
       <c r="H337">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="338">
@@ -9295,7 +9295,7 @@
         <v>PASS</v>
       </c>
       <c r="H338">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="339">
@@ -9321,7 +9321,7 @@
         <v>PASS</v>
       </c>
       <c r="H339">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="340">
@@ -9347,7 +9347,7 @@
         <v>PASS</v>
       </c>
       <c r="H340">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="341">
@@ -9373,7 +9373,7 @@
         <v>PASS</v>
       </c>
       <c r="H341">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="342">
@@ -9399,7 +9399,7 @@
         <v>PASS</v>
       </c>
       <c r="H342">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="343">
@@ -9425,7 +9425,7 @@
         <v>PASS</v>
       </c>
       <c r="H343">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="344">
@@ -9451,7 +9451,7 @@
         <v>PASS</v>
       </c>
       <c r="H344">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="345">
@@ -9477,7 +9477,7 @@
         <v>PASS</v>
       </c>
       <c r="H345">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="346">
@@ -9529,7 +9529,7 @@
         <v>PASS</v>
       </c>
       <c r="H347">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="348">
@@ -9555,7 +9555,7 @@
         <v>PASS</v>
       </c>
       <c r="H348">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="349">
@@ -9581,7 +9581,7 @@
         <v>PASS</v>
       </c>
       <c r="H349">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="350">
@@ -9607,7 +9607,7 @@
         <v>PASS</v>
       </c>
       <c r="H350">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="351">
@@ -9633,7 +9633,7 @@
         <v>PASS</v>
       </c>
       <c r="H351">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="352">
@@ -9659,7 +9659,7 @@
         <v>PASS</v>
       </c>
       <c r="H352">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="353">
@@ -9685,7 +9685,7 @@
         <v>PASS</v>
       </c>
       <c r="H353">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="354">
@@ -9711,7 +9711,7 @@
         <v>PASS</v>
       </c>
       <c r="H354">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="355">
@@ -9737,7 +9737,7 @@
         <v>PASS</v>
       </c>
       <c r="H355">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="356">
@@ -9763,7 +9763,7 @@
         <v>PASS</v>
       </c>
       <c r="H356">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="357">
@@ -9789,7 +9789,7 @@
         <v>PASS</v>
       </c>
       <c r="H357">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="358">
@@ -9815,7 +9815,7 @@
         <v>PASS</v>
       </c>
       <c r="H358">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="359">
@@ -9841,7 +9841,7 @@
         <v>PASS</v>
       </c>
       <c r="H359">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="360">
@@ -9893,7 +9893,7 @@
         <v>PASS</v>
       </c>
       <c r="H361">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="362">
@@ -9919,7 +9919,7 @@
         <v>PASS</v>
       </c>
       <c r="H362">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="363">
@@ -9945,7 +9945,7 @@
         <v>PASS</v>
       </c>
       <c r="H363">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="364">
@@ -9997,7 +9997,7 @@
         <v>PASS</v>
       </c>
       <c r="H365">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="366">
@@ -10049,7 +10049,7 @@
         <v>PASS</v>
       </c>
       <c r="H367">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="368">
@@ -10101,7 +10101,7 @@
         <v>PASS</v>
       </c>
       <c r="H369">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="370">
@@ -10127,7 +10127,7 @@
         <v>PASS</v>
       </c>
       <c r="H370">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="371">
@@ -10153,7 +10153,7 @@
         <v>PASS</v>
       </c>
       <c r="H371">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="372">
@@ -10231,7 +10231,7 @@
         <v>PASS</v>
       </c>
       <c r="H374">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="375">
@@ -10257,7 +10257,7 @@
         <v>PASS</v>
       </c>
       <c r="H375">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="376">
@@ -10283,7 +10283,7 @@
         <v>PASS</v>
       </c>
       <c r="H376">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="377">
@@ -10309,7 +10309,7 @@
         <v>PASS</v>
       </c>
       <c r="H377">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="378">
@@ -10335,7 +10335,7 @@
         <v>PASS</v>
       </c>
       <c r="H378">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="379">
@@ -10361,7 +10361,7 @@
         <v>PASS</v>
       </c>
       <c r="H379">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="380">
@@ -10387,7 +10387,7 @@
         <v>PASS</v>
       </c>
       <c r="H380">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="381">
@@ -10413,7 +10413,7 @@
         <v>PASS</v>
       </c>
       <c r="H381">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="382">
@@ -10439,7 +10439,7 @@
         <v>PASS</v>
       </c>
       <c r="H382">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="383">
@@ -10465,7 +10465,7 @@
         <v>PASS</v>
       </c>
       <c r="H383">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="384">
@@ -10491,7 +10491,7 @@
         <v>PASS</v>
       </c>
       <c r="H384">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="385">
@@ -10517,7 +10517,7 @@
         <v>PASS</v>
       </c>
       <c r="H385">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="386">
@@ -10543,7 +10543,7 @@
         <v>PASS</v>
       </c>
       <c r="H386">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="387">
@@ -10595,7 +10595,7 @@
         <v>PASS</v>
       </c>
       <c r="H388">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="389">
@@ -10647,7 +10647,7 @@
         <v>PASS</v>
       </c>
       <c r="H390">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="391">
@@ -10673,7 +10673,7 @@
         <v>PASS</v>
       </c>
       <c r="H391">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="392">
@@ -10699,7 +10699,7 @@
         <v>PASS</v>
       </c>
       <c r="H392">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="393">
@@ -10751,7 +10751,7 @@
         <v>PASS</v>
       </c>
       <c r="H394">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="395">
@@ -10777,7 +10777,7 @@
         <v>PASS</v>
       </c>
       <c r="H395">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="396">
@@ -10803,7 +10803,7 @@
         <v>PASS</v>
       </c>
       <c r="H396">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="397">
@@ -10855,7 +10855,7 @@
         <v>PASS</v>
       </c>
       <c r="H398">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="399">
@@ -10881,7 +10881,7 @@
         <v>PASS</v>
       </c>
       <c r="H399">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="400">
@@ -10907,7 +10907,7 @@
         <v>PASS</v>
       </c>
       <c r="H400">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="401">
@@ -10933,7 +10933,7 @@
         <v>PASS</v>
       </c>
       <c r="H401">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>